<commit_message>
feat(excel): enhance heatmap with top 5 risks list + polish (P2-4)
</commit_message>
<xml_diff>
--- a/examples/risk-register-aether-labs.xlsx
+++ b/examples/risk-register-aether-labs.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,8 +42,11 @@
       <b val="1"/>
       <sz val="14"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -80,6 +83,12 @@
         <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -93,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -104,6 +113,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2018,7 +2029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2161,6 +2172,185 @@
       <c r="A11" t="inlineStr">
         <is>
           <t>Total risks: 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Top 5 Risks (by inherent score)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Asset</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Threat</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>R-002</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Source code repository (GitHub)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Malicious code injection via compromised dependency</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>16</v>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>R-001</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Customer workspace database (RDS)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Unauthorized access / data breach</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>15</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>R-003</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CI/CD pipelines (GitHub Actions)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Supply chain attack on runner or action</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>15</v>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>R-018</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Secrets (GitHub + AWS)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Secret committed to repo</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>15</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>5</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>R-005</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Employee laptops / endpoints</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Phishing leading to credential theft + initial access</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>12</v>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>

</xml_diff>